<commit_message>
Add supapase into require
</commit_message>
<xml_diff>
--- a/Mẫu số đo & Đánh giá Model CV_THONGTHIEN.xlsx
+++ b/Mẫu số đo & Đánh giá Model CV_THONGTHIEN.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Lap_Trinh_2022-2026-20230924T092707Z-001\Bodyfat_predict\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{215BD6EB-30D7-40C4-B3FC-4131D3F7351B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94403E16-A5BF-4C95-8C16-E1EB0765FAA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-118" yWindow="-118" windowWidth="25370" windowHeight="13667" xr2:uid="{F2E29C3A-FB58-4893-8DD4-400619C0E675}"/>
   </bookViews>
@@ -287,7 +287,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
@@ -311,6 +311,7 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -371,8 +372,8 @@
       </xdr:blipFill>
       <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="3437146" y="1567192"/>
-          <a:ext cx="3013805" cy="4566432"/>
+          <a:off x="3430769" y="1527648"/>
+          <a:ext cx="3011253" cy="4484794"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1569,27 +1570,19 @@
       <c r="F44" s="11">
         <v>86</v>
       </c>
-      <c r="G44" s="12">
-        <v>88.62</v>
-      </c>
+      <c r="G44" s="12"/>
       <c r="H44" s="11">
         <v>74</v>
       </c>
-      <c r="I44" s="12">
-        <v>79.650000000000006</v>
-      </c>
+      <c r="I44" s="12"/>
       <c r="J44" s="11">
         <v>90</v>
       </c>
-      <c r="K44" s="12">
-        <v>91.32</v>
-      </c>
+      <c r="K44" s="12"/>
       <c r="L44" s="11">
         <v>50</v>
       </c>
-      <c r="M44" s="12">
-        <v>42.97</v>
-      </c>
+      <c r="M44" s="12"/>
     </row>
     <row r="45" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A45" s="11">
@@ -1610,27 +1603,19 @@
       <c r="F45" s="11">
         <v>89</v>
       </c>
-      <c r="G45" s="12">
-        <v>106.69</v>
-      </c>
+      <c r="G45" s="12"/>
       <c r="H45" s="11">
         <v>73</v>
       </c>
-      <c r="I45" s="12">
-        <v>80.61</v>
-      </c>
+      <c r="I45" s="12"/>
       <c r="J45" s="11">
         <v>86</v>
       </c>
-      <c r="K45" s="12">
-        <v>89.53</v>
-      </c>
+      <c r="K45" s="12"/>
       <c r="L45" s="11">
         <v>48</v>
       </c>
-      <c r="M45" s="12">
-        <v>37.01</v>
-      </c>
+      <c r="M45" s="12"/>
     </row>
     <row r="46" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A46" s="11">
@@ -1651,68 +1636,52 @@
       <c r="F46" s="11">
         <v>83</v>
       </c>
-      <c r="G46" s="12">
-        <v>103.19</v>
-      </c>
+      <c r="G46" s="12"/>
       <c r="H46" s="11">
         <v>69</v>
       </c>
-      <c r="I46" s="12">
-        <v>82.35</v>
-      </c>
+      <c r="I46" s="12"/>
       <c r="J46" s="11">
         <v>85</v>
       </c>
-      <c r="K46" s="12">
-        <v>92.72</v>
-      </c>
+      <c r="K46" s="12"/>
       <c r="L46" s="11">
         <v>48</v>
       </c>
-      <c r="M46" s="12">
-        <v>55.05</v>
-      </c>
+      <c r="M46" s="12"/>
     </row>
     <row r="47" spans="1:26" x14ac:dyDescent="0.3">
-      <c r="A47" s="14">
+      <c r="A47" s="9">
         <v>4</v>
       </c>
-      <c r="B47" s="15" t="s">
+      <c r="B47" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="C47" s="14">
+      <c r="C47" s="9">
         <v>167</v>
       </c>
-      <c r="D47" s="14">
+      <c r="D47" s="9">
         <v>64</v>
       </c>
-      <c r="E47" s="14">
+      <c r="E47" s="9">
         <v>22</v>
       </c>
-      <c r="F47" s="14">
+      <c r="F47" s="9">
         <v>90</v>
       </c>
-      <c r="G47" s="16">
-        <v>94.72</v>
-      </c>
-      <c r="H47" s="14">
+      <c r="G47" s="17"/>
+      <c r="H47" s="9">
         <v>84</v>
       </c>
-      <c r="I47" s="16">
-        <v>81.28</v>
-      </c>
-      <c r="J47" s="14">
+      <c r="I47" s="17"/>
+      <c r="J47" s="9">
         <v>93</v>
       </c>
-      <c r="K47" s="16">
-        <v>98.56</v>
-      </c>
-      <c r="L47" s="14">
+      <c r="K47" s="17"/>
+      <c r="L47" s="9">
         <v>46</v>
       </c>
-      <c r="M47" s="16">
-        <v>55.04</v>
-      </c>
+      <c r="M47" s="17"/>
     </row>
     <row r="48" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A48" s="11">
@@ -1733,29 +1702,21 @@
       <c r="F48" s="11">
         <v>90</v>
       </c>
-      <c r="G48" s="12">
-        <v>101.5</v>
-      </c>
+      <c r="G48" s="12"/>
       <c r="H48" s="11">
         <v>75</v>
       </c>
-      <c r="I48" s="12">
-        <v>74.53</v>
-      </c>
+      <c r="I48" s="12"/>
       <c r="J48" s="11">
         <v>86</v>
       </c>
-      <c r="K48" s="12">
-        <v>82.12</v>
-      </c>
+      <c r="K48" s="12"/>
       <c r="L48" s="11">
         <v>52</v>
       </c>
-      <c r="M48" s="12">
-        <v>32.090000000000003</v>
-      </c>
-    </row>
-    <row r="49" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="M48" s="12"/>
+    </row>
+    <row r="49" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A49" s="11">
         <v>6</v>
       </c>
@@ -1786,14 +1747,14 @@
       <c r="L49" s="11">
         <v>51</v>
       </c>
-      <c r="M49" s="11"/>
-    </row>
-    <row r="60" spans="1:13" ht="15.75" x14ac:dyDescent="0.3">
+      <c r="N49" s="11"/>
+    </row>
+    <row r="60" spans="1:14" ht="15.75" x14ac:dyDescent="0.3">
       <c r="B60" s="8" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="61" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A61" s="11" t="s">
         <v>0</v>
       </c>
@@ -1807,7 +1768,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="62" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A62" s="11">
         <v>1</v>
       </c>
@@ -1817,7 +1778,7 @@
       <c r="C62" s="11"/>
       <c r="D62" s="11"/>
     </row>
-    <row r="63" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A63" s="11">
         <v>2</v>
       </c>
@@ -1827,7 +1788,7 @@
       <c r="C63" s="11"/>
       <c r="D63" s="11"/>
     </row>
-    <row r="64" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A64" s="11">
         <v>3</v>
       </c>

</xml_diff>

<commit_message>
Them file calibration de tinh f_bmi avg, test_all_tabs de chay toan bo file anh qua 3 tab
</commit_message>
<xml_diff>
--- a/Mẫu số đo & Đánh giá Model CV_THONGTHIEN.xlsx
+++ b/Mẫu số đo & Đánh giá Model CV_THONGTHIEN.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Lap_Trinh_2022-2026-20230924T092707Z-001\Bodyfat_predict\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94403E16-A5BF-4C95-8C16-E1EB0765FAA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91902ECF-9515-49E7-ACC5-E19C5FA4D862}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-118" yWindow="-118" windowWidth="25370" windowHeight="13667" xr2:uid="{F2E29C3A-FB58-4893-8DD4-400619C0E675}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="24">
   <si>
     <t>STT</t>
   </si>
@@ -173,45 +173,6 @@
   </si>
   <si>
     <t>Ảnh lỗi nặng</t>
-  </si>
-  <si>
-    <t>Bảng 1: Sai số của AI Scan</t>
-  </si>
-  <si>
-    <t>Không</t>
-  </si>
-  <si>
-    <t>Bảng 2: Sai số của mô hình ML (Nhập/ Scan)</t>
-  </si>
-  <si>
-    <t>Nhập</t>
-  </si>
-  <si>
-    <t>Scan</t>
-  </si>
-  <si>
-    <t>Nếu mô hình dự đoán tốt với số đo thực tế nhưng kém với số đo từ ảnh, thì vấn đề chính là ở CV chứ không phải XGBoost.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bổ sung ngay phần “hướng dẫn người dùng chụp ảnh chuẩn” + đưa lên web hướng dẫn người dùng </t>
-  </si>
-  <si>
-    <t>Bảng 3: Bảng so sánh hệ số trong công thức pixel -&gt; cm</t>
-  </si>
-  <si>
-    <t>Hệ số</t>
-  </si>
-  <si>
-    <t>cm</t>
-  </si>
-  <si>
-    <t>scan</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mũi -&gt; mắt x hệ số = mũi -&gt; đầu ; =&gt; vị trí đỉnh đầu </t>
-  </si>
-  <si>
-    <t>Bảng 4: Tối ưu lại phần quét biên và xử lý quần áo rộng</t>
   </si>
 </sst>
 </file>
@@ -287,7 +248,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
@@ -311,7 +272,8 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1139,7 +1101,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9567F0BA-FA29-4B5F-8970-6B09AC94066C}">
-  <dimension ref="A1:Z93"/>
+  <dimension ref="A1:Z87"/>
   <sheetFormatPr defaultRowHeight="15.05" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.33203125" customWidth="1"/>
@@ -1505,500 +1467,294 @@
       <c r="Y41" s="7"/>
       <c r="Z41" s="7"/>
     </row>
-    <row r="42" spans="1:26" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="B42" s="8" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="43" spans="1:26" x14ac:dyDescent="0.3">
-      <c r="A43" s="11" t="s">
-        <v>0</v>
-      </c>
-      <c r="B43" s="11" t="s">
-        <v>1</v>
-      </c>
-      <c r="C43" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="D43" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="E43" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="F43" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="G43" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="H43" s="11" t="s">
-        <v>2</v>
-      </c>
-      <c r="I43" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="J43" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="K43" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="L43" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="M43" s="12" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="44" spans="1:26" x14ac:dyDescent="0.3">
-      <c r="A44" s="11">
-        <v>1</v>
-      </c>
-      <c r="B44" s="13" t="s">
-        <v>6</v>
-      </c>
-      <c r="C44" s="11">
-        <v>169</v>
-      </c>
-      <c r="D44" s="11">
-        <v>59</v>
-      </c>
-      <c r="E44" s="11">
-        <v>22</v>
-      </c>
-      <c r="F44" s="11">
-        <v>86</v>
-      </c>
-      <c r="G44" s="12"/>
-      <c r="H44" s="11">
-        <v>74</v>
-      </c>
-      <c r="I44" s="12"/>
-      <c r="J44" s="11">
-        <v>90</v>
-      </c>
-      <c r="K44" s="12"/>
-      <c r="L44" s="11">
-        <v>50</v>
-      </c>
-      <c r="M44" s="12"/>
-    </row>
     <row r="45" spans="1:26" x14ac:dyDescent="0.3">
-      <c r="A45" s="11">
-        <v>2</v>
-      </c>
-      <c r="B45" s="13" t="s">
-        <v>8</v>
-      </c>
-      <c r="C45" s="11">
-        <v>163</v>
-      </c>
-      <c r="D45" s="11">
-        <v>61</v>
-      </c>
-      <c r="E45" s="11">
-        <v>22</v>
-      </c>
-      <c r="F45" s="11">
-        <v>89</v>
-      </c>
-      <c r="G45" s="12"/>
-      <c r="H45" s="11">
-        <v>73</v>
-      </c>
-      <c r="I45" s="12"/>
-      <c r="J45" s="11">
-        <v>86</v>
-      </c>
-      <c r="K45" s="12"/>
-      <c r="L45" s="11">
-        <v>48</v>
-      </c>
-      <c r="M45" s="12"/>
+      <c r="G45" s="17"/>
+      <c r="H45" s="18"/>
+      <c r="I45" s="17"/>
+      <c r="J45" s="17"/>
+      <c r="K45" s="17"/>
     </row>
     <row r="46" spans="1:26" x14ac:dyDescent="0.3">
-      <c r="A46" s="11">
-        <v>3</v>
-      </c>
-      <c r="B46" s="13" t="s">
-        <v>9</v>
-      </c>
-      <c r="C46" s="11">
-        <v>176</v>
-      </c>
-      <c r="D46" s="11">
-        <v>60</v>
-      </c>
-      <c r="E46" s="11">
-        <v>22</v>
-      </c>
-      <c r="F46" s="11">
-        <v>83</v>
-      </c>
-      <c r="G46" s="12"/>
-      <c r="H46" s="11">
-        <v>69</v>
-      </c>
-      <c r="I46" s="12"/>
-      <c r="J46" s="11">
-        <v>85</v>
-      </c>
-      <c r="K46" s="12"/>
-      <c r="L46" s="11">
-        <v>48</v>
-      </c>
-      <c r="M46" s="12"/>
+      <c r="G46" s="17"/>
+      <c r="H46" s="17"/>
+      <c r="I46" s="17"/>
+      <c r="J46" s="17"/>
+      <c r="K46" s="17"/>
     </row>
     <row r="47" spans="1:26" x14ac:dyDescent="0.3">
-      <c r="A47" s="9">
-        <v>4</v>
-      </c>
-      <c r="B47" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="C47" s="9">
-        <v>167</v>
-      </c>
-      <c r="D47" s="9">
-        <v>64</v>
-      </c>
-      <c r="E47" s="9">
-        <v>22</v>
-      </c>
-      <c r="F47" s="9">
-        <v>90</v>
-      </c>
       <c r="G47" s="17"/>
-      <c r="H47" s="9">
-        <v>84</v>
-      </c>
+      <c r="H47" s="17"/>
       <c r="I47" s="17"/>
-      <c r="J47" s="9">
-        <v>93</v>
-      </c>
+      <c r="J47" s="17"/>
       <c r="K47" s="17"/>
-      <c r="L47" s="9">
-        <v>46</v>
-      </c>
-      <c r="M47" s="17"/>
     </row>
     <row r="48" spans="1:26" x14ac:dyDescent="0.3">
-      <c r="A48" s="11">
-        <v>5</v>
-      </c>
-      <c r="B48" s="13" t="s">
-        <v>7</v>
-      </c>
-      <c r="C48" s="11">
-        <v>158</v>
-      </c>
-      <c r="D48" s="11">
-        <v>58</v>
-      </c>
-      <c r="E48" s="11">
-        <v>22</v>
-      </c>
-      <c r="F48" s="11">
-        <v>90</v>
-      </c>
-      <c r="G48" s="12"/>
-      <c r="H48" s="11">
-        <v>75</v>
-      </c>
-      <c r="I48" s="12"/>
-      <c r="J48" s="11">
-        <v>86</v>
-      </c>
-      <c r="K48" s="12"/>
-      <c r="L48" s="11">
-        <v>52</v>
-      </c>
-      <c r="M48" s="12"/>
-    </row>
-    <row r="49" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A49" s="11">
-        <v>6</v>
-      </c>
-      <c r="B49" s="13" t="s">
-        <v>25</v>
-      </c>
-      <c r="C49" s="11">
-        <v>165</v>
-      </c>
-      <c r="D49" s="11">
-        <v>51</v>
-      </c>
-      <c r="E49" s="11">
-        <v>18</v>
-      </c>
-      <c r="F49" s="11">
-        <v>81</v>
-      </c>
-      <c r="G49" s="11"/>
-      <c r="H49" s="11">
-        <v>67</v>
-      </c>
-      <c r="I49" s="11"/>
-      <c r="J49" s="11">
-        <v>95</v>
-      </c>
-      <c r="K49" s="11"/>
-      <c r="L49" s="11">
-        <v>51</v>
-      </c>
-      <c r="N49" s="11"/>
-    </row>
-    <row r="60" spans="1:14" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="B60" s="8" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="61" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A61" s="11" t="s">
-        <v>0</v>
-      </c>
-      <c r="B61" s="11" t="s">
-        <v>1</v>
-      </c>
-      <c r="C61" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="D61" s="11" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="62" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A62" s="11">
-        <v>1</v>
-      </c>
-      <c r="B62" s="13" t="s">
-        <v>6</v>
-      </c>
-      <c r="C62" s="11"/>
-      <c r="D62" s="11"/>
-    </row>
-    <row r="63" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A63" s="11">
-        <v>2</v>
-      </c>
-      <c r="B63" s="13" t="s">
-        <v>8</v>
-      </c>
+      <c r="G48" s="17"/>
+      <c r="H48" s="17"/>
+      <c r="I48" s="17"/>
+      <c r="J48" s="17"/>
+      <c r="K48" s="17"/>
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="G49" s="17"/>
+      <c r="H49" s="17"/>
+      <c r="I49" s="17"/>
+      <c r="J49" s="17"/>
+      <c r="K49" s="17"/>
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="G50" s="17"/>
+      <c r="H50" s="17"/>
+      <c r="I50" s="17"/>
+      <c r="J50" s="17"/>
+      <c r="K50" s="17"/>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A51" s="17"/>
+      <c r="B51" s="18"/>
+      <c r="C51" s="17"/>
+      <c r="D51" s="17"/>
+      <c r="E51" s="17"/>
+      <c r="F51" s="17"/>
+      <c r="G51" s="17"/>
+      <c r="H51" s="17"/>
+      <c r="I51" s="17"/>
+      <c r="J51" s="17"/>
+      <c r="K51" s="17"/>
+    </row>
+    <row r="53" spans="1:11" ht="15.75" x14ac:dyDescent="0.3">
+      <c r="B53" s="8"/>
+    </row>
+    <row r="54" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A54" s="11"/>
+      <c r="B54" s="11"/>
+      <c r="C54" s="11"/>
+      <c r="D54" s="11"/>
+      <c r="E54" s="11"/>
+      <c r="F54" s="13"/>
+      <c r="G54" s="13"/>
+      <c r="H54" s="13"/>
+      <c r="I54" s="10"/>
+      <c r="J54" s="13"/>
+      <c r="K54" s="13"/>
+    </row>
+    <row r="55" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A55" s="11"/>
+      <c r="B55" s="11"/>
+      <c r="C55" s="11"/>
+      <c r="D55" s="11"/>
+      <c r="E55" s="11"/>
+      <c r="F55" s="11"/>
+      <c r="G55" s="11"/>
+      <c r="H55" s="11"/>
+      <c r="I55" s="11"/>
+      <c r="J55" s="11"/>
+      <c r="K55" s="11"/>
+    </row>
+    <row r="56" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A56" s="11"/>
+      <c r="B56" s="13"/>
+      <c r="C56" s="11"/>
+      <c r="D56" s="11"/>
+      <c r="E56" s="11"/>
+      <c r="F56" s="11"/>
+      <c r="G56" s="11"/>
+      <c r="H56" s="11"/>
+      <c r="I56" s="11"/>
+      <c r="J56" s="11"/>
+      <c r="K56" s="11"/>
+    </row>
+    <row r="57" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A57" s="11"/>
+      <c r="B57" s="13"/>
+      <c r="C57" s="11"/>
+      <c r="D57" s="11"/>
+      <c r="E57" s="11"/>
+      <c r="F57" s="11"/>
+      <c r="G57" s="11"/>
+      <c r="H57" s="11"/>
+      <c r="I57" s="11"/>
+      <c r="J57" s="11"/>
+      <c r="K57" s="11"/>
+    </row>
+    <row r="58" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A58" s="9"/>
+      <c r="B58" s="10"/>
+      <c r="C58" s="9"/>
+      <c r="D58" s="9"/>
+      <c r="E58" s="11"/>
+      <c r="F58" s="11"/>
+      <c r="G58" s="11"/>
+      <c r="H58" s="11"/>
+      <c r="I58" s="11"/>
+      <c r="J58" s="11"/>
+      <c r="K58" s="11"/>
+    </row>
+    <row r="59" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A59" s="11"/>
+      <c r="B59" s="13"/>
+      <c r="C59" s="11"/>
+      <c r="D59" s="11"/>
+      <c r="E59" s="11"/>
+      <c r="F59" s="11"/>
+      <c r="G59" s="11"/>
+      <c r="H59" s="11"/>
+      <c r="I59" s="11"/>
+      <c r="J59" s="11"/>
+      <c r="K59" s="11"/>
+    </row>
+    <row r="60" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A60" s="11"/>
+      <c r="B60" s="13"/>
+      <c r="C60" s="11"/>
+      <c r="D60" s="11"/>
+      <c r="E60" s="11"/>
+      <c r="F60" s="11"/>
+      <c r="G60" s="11"/>
+      <c r="H60" s="11"/>
+      <c r="I60" s="11"/>
+      <c r="J60" s="11"/>
+      <c r="K60" s="11"/>
+    </row>
+    <row r="62" spans="1:11" ht="15.75" x14ac:dyDescent="0.3">
+      <c r="B62" s="8"/>
+    </row>
+    <row r="63" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A63" s="11"/>
+      <c r="B63" s="11"/>
       <c r="C63" s="11"/>
       <c r="D63" s="11"/>
-    </row>
-    <row r="64" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A64" s="11">
-        <v>3</v>
-      </c>
-      <c r="B64" s="13" t="s">
-        <v>9</v>
-      </c>
+      <c r="E63" s="11"/>
+      <c r="F63" s="13"/>
+      <c r="G63" s="13"/>
+      <c r="H63" s="13"/>
+      <c r="I63" s="10"/>
+      <c r="J63" s="13"/>
+      <c r="K63" s="13"/>
+    </row>
+    <row r="64" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A64" s="11"/>
+      <c r="B64" s="11"/>
       <c r="C64" s="11"/>
       <c r="D64" s="11"/>
-    </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A65" s="9">
-        <v>4</v>
-      </c>
-      <c r="B65" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="C65" s="9"/>
-      <c r="D65" s="9"/>
-    </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A66" s="11">
-        <v>5</v>
-      </c>
-      <c r="B66" s="13" t="s">
-        <v>7</v>
-      </c>
+      <c r="E64" s="11"/>
+      <c r="F64" s="11"/>
+      <c r="G64" s="11"/>
+      <c r="H64" s="11"/>
+      <c r="I64" s="11"/>
+      <c r="J64" s="11"/>
+      <c r="K64" s="11"/>
+    </row>
+    <row r="65" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A65" s="11"/>
+      <c r="B65" s="13"/>
+      <c r="C65" s="11"/>
+      <c r="D65" s="11"/>
+      <c r="E65" s="11"/>
+      <c r="F65" s="11"/>
+      <c r="G65" s="11"/>
+      <c r="H65" s="11"/>
+      <c r="I65" s="11"/>
+      <c r="J65" s="11"/>
+      <c r="K65" s="11"/>
+    </row>
+    <row r="66" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A66" s="11"/>
+      <c r="B66" s="13"/>
       <c r="C66" s="11"/>
       <c r="D66" s="11"/>
-    </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A67" s="11">
-        <v>6</v>
-      </c>
-      <c r="B67" s="13" t="s">
-        <v>25</v>
-      </c>
-      <c r="C67" s="11"/>
-      <c r="D67" s="11"/>
-    </row>
-    <row r="69" spans="1:4" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A69" s="8" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="70" spans="1:4" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="A70" s="8" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="81" spans="1:11" ht="15.75" x14ac:dyDescent="0.3">
-      <c r="B81" s="8" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A82" s="11" t="s">
-        <v>0</v>
-      </c>
-      <c r="B82" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="C82" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="D82" s="11" t="s">
-        <v>32</v>
-      </c>
-      <c r="E82" s="11" t="s">
-        <v>34</v>
-      </c>
-      <c r="F82" s="13" t="s">
-        <v>6</v>
-      </c>
-      <c r="G82" s="13" t="s">
-        <v>8</v>
-      </c>
-      <c r="H82" s="13" t="s">
-        <v>9</v>
-      </c>
-      <c r="I82" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="J82" s="13" t="s">
-        <v>7</v>
-      </c>
-      <c r="K82" s="13" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="83" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A83" s="11">
-        <v>1</v>
-      </c>
-      <c r="B83" s="11">
-        <v>1</v>
-      </c>
-      <c r="C83" s="11">
-        <v>169</v>
-      </c>
+      <c r="E66" s="11"/>
+      <c r="F66" s="11"/>
+      <c r="G66" s="11"/>
+      <c r="H66" s="11"/>
+      <c r="I66" s="11"/>
+      <c r="J66" s="11"/>
+      <c r="K66" s="11"/>
+    </row>
+    <row r="67" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A67" s="9"/>
+      <c r="B67" s="10"/>
+      <c r="C67" s="9"/>
+      <c r="D67" s="9"/>
+      <c r="E67" s="11"/>
+      <c r="F67" s="11"/>
+      <c r="G67" s="11"/>
+      <c r="H67" s="11"/>
+      <c r="I67" s="11"/>
+      <c r="J67" s="11"/>
+      <c r="K67" s="11"/>
+    </row>
+    <row r="68" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A68" s="11"/>
+      <c r="B68" s="13"/>
+      <c r="C68" s="11"/>
+      <c r="D68" s="11"/>
+      <c r="E68" s="11"/>
+      <c r="F68" s="11"/>
+      <c r="G68" s="11"/>
+      <c r="H68" s="11"/>
+      <c r="I68" s="11"/>
+      <c r="J68" s="11"/>
+      <c r="K68" s="11"/>
+    </row>
+    <row r="69" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A69" s="11"/>
+      <c r="B69" s="13"/>
+      <c r="C69" s="11"/>
+      <c r="D69" s="11"/>
+      <c r="E69" s="11"/>
+      <c r="F69" s="11"/>
+      <c r="G69" s="11"/>
+      <c r="H69" s="11"/>
+      <c r="I69" s="11"/>
+      <c r="J69" s="11"/>
+      <c r="K69" s="11"/>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A81" s="11"/>
+      <c r="B81" s="11"/>
+      <c r="C81" s="11"/>
+      <c r="D81" s="11"/>
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A82" s="11"/>
+      <c r="B82" s="13"/>
+      <c r="C82" s="11"/>
+      <c r="D82" s="11"/>
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A83" s="11"/>
+      <c r="B83" s="13"/>
+      <c r="C83" s="11"/>
       <c r="D83" s="11"/>
-      <c r="E83" s="11"/>
-      <c r="F83" s="11"/>
-      <c r="G83" s="11"/>
-      <c r="H83" s="11"/>
-      <c r="I83" s="11"/>
-      <c r="J83" s="11"/>
-      <c r="K83" s="11"/>
-    </row>
-    <row r="84" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A84" s="11">
-        <v>2</v>
-      </c>
-      <c r="B84" s="13">
-        <v>3</v>
-      </c>
-      <c r="C84" s="11">
-        <v>163</v>
-      </c>
+    </row>
+    <row r="84" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A84" s="11"/>
+      <c r="B84" s="13"/>
+      <c r="C84" s="11"/>
       <c r="D84" s="11"/>
-      <c r="E84" s="11"/>
-      <c r="F84" s="11"/>
-      <c r="G84" s="11"/>
-      <c r="H84" s="11"/>
-      <c r="I84" s="11"/>
-      <c r="J84" s="11"/>
-      <c r="K84" s="11"/>
-    </row>
-    <row r="85" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A85" s="11">
-        <v>3</v>
-      </c>
-      <c r="B85" s="13">
-        <v>2</v>
-      </c>
-      <c r="C85" s="11">
-        <v>176</v>
-      </c>
-      <c r="D85" s="11"/>
-      <c r="E85" s="11"/>
-      <c r="F85" s="11"/>
-      <c r="G85" s="11"/>
-      <c r="H85" s="11"/>
-      <c r="I85" s="11"/>
-      <c r="J85" s="11"/>
-      <c r="K85" s="11"/>
-    </row>
-    <row r="86" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A86" s="9">
-        <v>4</v>
-      </c>
-      <c r="B86" s="10">
-        <v>4</v>
-      </c>
-      <c r="C86" s="9">
-        <v>167</v>
-      </c>
-      <c r="D86" s="9"/>
-      <c r="E86" s="11"/>
-      <c r="F86" s="11"/>
-      <c r="G86" s="11"/>
-      <c r="H86" s="11"/>
-      <c r="I86" s="11"/>
-      <c r="J86" s="11"/>
-      <c r="K86" s="11"/>
-    </row>
-    <row r="87" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A87" s="11">
-        <v>5</v>
-      </c>
-      <c r="B87" s="13">
-        <v>5</v>
-      </c>
-      <c r="C87" s="11">
-        <v>158</v>
-      </c>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A85" s="9"/>
+      <c r="B85" s="10"/>
+      <c r="C85" s="9"/>
+      <c r="D85" s="9"/>
+    </row>
+    <row r="86" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A86" s="11"/>
+      <c r="B86" s="13"/>
+      <c r="C86" s="11"/>
+      <c r="D86" s="11"/>
+    </row>
+    <row r="87" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A87" s="11"/>
+      <c r="B87" s="13"/>
+      <c r="C87" s="11"/>
       <c r="D87" s="11"/>
-      <c r="E87" s="11"/>
-      <c r="F87" s="11"/>
-      <c r="G87" s="11"/>
-      <c r="H87" s="11"/>
-      <c r="I87" s="11"/>
-      <c r="J87" s="11"/>
-      <c r="K87" s="11"/>
-    </row>
-    <row r="88" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A88" s="11">
-        <v>6</v>
-      </c>
-      <c r="B88" s="13">
-        <v>6</v>
-      </c>
-      <c r="C88" s="11">
-        <v>165</v>
-      </c>
-      <c r="D88" s="11"/>
-      <c r="E88" s="11"/>
-      <c r="F88" s="11"/>
-      <c r="G88" s="11"/>
-      <c r="H88" s="11"/>
-      <c r="I88" s="11"/>
-      <c r="J88" s="11"/>
-      <c r="K88" s="11"/>
-    </row>
-    <row r="93" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B93" t="s">
-        <v>36</v>
-      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>